<commit_message>
some changes are made in seed file
</commit_message>
<xml_diff>
--- a/db/data/office_items.xlsx
+++ b/db/data/office_items.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pradeep\Desktop\storemgmt\db\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1499A608-33F4-4C7A-93B4-A9298D88A21C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2BA0712-B91A-4C7D-A23A-C633F689A677}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2276,7 +2276,7 @@
         <v>5</v>
       </c>
       <c r="F2">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -2293,7 +2293,7 @@
         <v>7</v>
       </c>
       <c r="F3">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -2310,7 +2310,7 @@
         <v>9</v>
       </c>
       <c r="F4">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -2327,7 +2327,7 @@
         <v>11</v>
       </c>
       <c r="F5">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2344,7 +2344,7 @@
         <v>13</v>
       </c>
       <c r="F6">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2361,7 +2361,7 @@
         <v>15</v>
       </c>
       <c r="F7">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2378,7 +2378,7 @@
         <v>17</v>
       </c>
       <c r="F8">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2395,7 +2395,7 @@
         <v>19</v>
       </c>
       <c r="F9">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2412,7 +2412,7 @@
         <v>21</v>
       </c>
       <c r="F10">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2429,7 +2429,7 @@
         <v>23</v>
       </c>
       <c r="F11">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2446,7 +2446,7 @@
         <v>25</v>
       </c>
       <c r="F12">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2463,7 +2463,7 @@
         <v>27</v>
       </c>
       <c r="F13">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -2480,7 +2480,7 @@
         <v>29</v>
       </c>
       <c r="F14">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -2497,7 +2497,7 @@
         <v>31</v>
       </c>
       <c r="F15">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -2514,7 +2514,7 @@
         <v>33</v>
       </c>
       <c r="F16">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
@@ -2531,7 +2531,7 @@
         <v>35</v>
       </c>
       <c r="F17">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.25">
@@ -2548,7 +2548,7 @@
         <v>37</v>
       </c>
       <c r="F18">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.25">
@@ -2565,7 +2565,7 @@
         <v>39</v>
       </c>
       <c r="F19">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
@@ -2582,7 +2582,7 @@
         <v>41</v>
       </c>
       <c r="F20">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.25">
@@ -2599,7 +2599,7 @@
         <v>43</v>
       </c>
       <c r="F21">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
@@ -2616,7 +2616,7 @@
         <v>45</v>
       </c>
       <c r="F22">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.25">
@@ -2633,7 +2633,7 @@
         <v>47</v>
       </c>
       <c r="F23">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.25">
@@ -2650,7 +2650,7 @@
         <v>49</v>
       </c>
       <c r="F24">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.25">
@@ -2667,7 +2667,7 @@
         <v>51</v>
       </c>
       <c r="F25">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.25">
@@ -2684,7 +2684,7 @@
         <v>53</v>
       </c>
       <c r="F26">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
@@ -2701,7 +2701,7 @@
         <v>55</v>
       </c>
       <c r="F27">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.25">
@@ -2718,7 +2718,7 @@
         <v>57</v>
       </c>
       <c r="F28">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
@@ -2735,7 +2735,7 @@
         <v>59</v>
       </c>
       <c r="F29">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
@@ -2752,7 +2752,7 @@
         <v>395</v>
       </c>
       <c r="F30">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
@@ -2769,7 +2769,7 @@
         <v>61</v>
       </c>
       <c r="F31">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -2786,7 +2786,7 @@
         <v>63</v>
       </c>
       <c r="F32">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
@@ -2803,7 +2803,7 @@
         <v>65</v>
       </c>
       <c r="F33">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.25">
@@ -2820,7 +2820,7 @@
         <v>67</v>
       </c>
       <c r="F34">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="35" spans="2:6" x14ac:dyDescent="0.25">
@@ -2837,7 +2837,7 @@
         <v>69</v>
       </c>
       <c r="F35">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
@@ -2854,7 +2854,7 @@
         <v>71</v>
       </c>
       <c r="F36">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
@@ -2871,7 +2871,7 @@
         <v>73</v>
       </c>
       <c r="F37">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
@@ -2888,7 +2888,7 @@
         <v>75</v>
       </c>
       <c r="F38">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
@@ -2905,7 +2905,7 @@
         <v>77</v>
       </c>
       <c r="F39">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
@@ -2922,7 +2922,7 @@
         <v>79</v>
       </c>
       <c r="F40">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
@@ -2939,7 +2939,7 @@
         <v>81</v>
       </c>
       <c r="F41">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
@@ -2956,7 +2956,7 @@
         <v>83</v>
       </c>
       <c r="F42">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
@@ -2973,7 +2973,7 @@
         <v>85</v>
       </c>
       <c r="F43">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
@@ -2990,7 +2990,7 @@
         <v>87</v>
       </c>
       <c r="F44">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.25">
@@ -3007,7 +3007,7 @@
         <v>89</v>
       </c>
       <c r="F45">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.25">
@@ -3024,7 +3024,7 @@
         <v>91</v>
       </c>
       <c r="F46">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="47" spans="2:6" x14ac:dyDescent="0.25">
@@ -3041,7 +3041,7 @@
         <v>93</v>
       </c>
       <c r="F47">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.25">
@@ -3058,7 +3058,7 @@
         <v>95</v>
       </c>
       <c r="F48">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.25">
@@ -3075,7 +3075,7 @@
         <v>97</v>
       </c>
       <c r="F49">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="50" spans="2:6" x14ac:dyDescent="0.25">
@@ -3092,7 +3092,7 @@
         <v>99</v>
       </c>
       <c r="F50">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.25">
@@ -3109,7 +3109,7 @@
         <v>101</v>
       </c>
       <c r="F51">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.25">
@@ -3126,7 +3126,7 @@
         <v>103</v>
       </c>
       <c r="F52">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.25">
@@ -3143,7 +3143,7 @@
         <v>105</v>
       </c>
       <c r="F53">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.25">
@@ -3160,7 +3160,7 @@
         <v>47</v>
       </c>
       <c r="F54">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="55" spans="2:6" x14ac:dyDescent="0.25">
@@ -3177,7 +3177,7 @@
         <v>107</v>
       </c>
       <c r="F55">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="56" spans="2:6" x14ac:dyDescent="0.25">
@@ -3194,7 +3194,7 @@
         <v>109</v>
       </c>
       <c r="F56">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="57" spans="2:6" x14ac:dyDescent="0.25">
@@ -3211,7 +3211,7 @@
         <v>111</v>
       </c>
       <c r="F57">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="58" spans="2:6" x14ac:dyDescent="0.25">
@@ -3228,7 +3228,7 @@
         <v>113</v>
       </c>
       <c r="F58">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="59" spans="2:6" x14ac:dyDescent="0.25">
@@ -3245,7 +3245,7 @@
         <v>115</v>
       </c>
       <c r="F59">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="60" spans="2:6" x14ac:dyDescent="0.25">
@@ -3262,7 +3262,7 @@
         <v>117</v>
       </c>
       <c r="F60">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="61" spans="2:6" x14ac:dyDescent="0.25">
@@ -3279,7 +3279,7 @@
         <v>119</v>
       </c>
       <c r="F61">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="62" spans="2:6" x14ac:dyDescent="0.25">
@@ -3296,7 +3296,7 @@
         <v>121</v>
       </c>
       <c r="F62">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="63" spans="2:6" x14ac:dyDescent="0.25">
@@ -3313,7 +3313,7 @@
         <v>123</v>
       </c>
       <c r="F63">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="64" spans="2:6" x14ac:dyDescent="0.25">
@@ -3330,7 +3330,7 @@
         <v>125</v>
       </c>
       <c r="F64">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.25">
@@ -3347,7 +3347,7 @@
         <v>127</v>
       </c>
       <c r="F65">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.25">
@@ -3364,7 +3364,7 @@
         <v>129</v>
       </c>
       <c r="F66">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="67" spans="2:6" x14ac:dyDescent="0.25">
@@ -3381,7 +3381,7 @@
         <v>131</v>
       </c>
       <c r="F67">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.25">
@@ -3398,7 +3398,7 @@
         <v>133</v>
       </c>
       <c r="F68">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="69" spans="2:6" x14ac:dyDescent="0.25">
@@ -3415,7 +3415,7 @@
         <v>135</v>
       </c>
       <c r="F69">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.25">
@@ -3432,7 +3432,7 @@
         <v>137</v>
       </c>
       <c r="F70">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="71" spans="2:6" x14ac:dyDescent="0.25">
@@ -3449,7 +3449,7 @@
         <v>139</v>
       </c>
       <c r="F71">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.25">
@@ -3466,7 +3466,7 @@
         <v>141</v>
       </c>
       <c r="F72">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="73" spans="2:6" x14ac:dyDescent="0.25">
@@ -3483,7 +3483,7 @@
         <v>143</v>
       </c>
       <c r="F73">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.25">
@@ -3500,7 +3500,7 @@
         <v>145</v>
       </c>
       <c r="F74">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="75" spans="2:6" x14ac:dyDescent="0.25">
@@ -3517,7 +3517,7 @@
         <v>147</v>
       </c>
       <c r="F75">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.25">
@@ -3534,7 +3534,7 @@
         <v>149</v>
       </c>
       <c r="F76">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.25">
@@ -3551,7 +3551,7 @@
         <v>151</v>
       </c>
       <c r="F77">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="78" spans="2:6" x14ac:dyDescent="0.25">
@@ -3568,7 +3568,7 @@
         <v>153</v>
       </c>
       <c r="F78">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="79" spans="2:6" x14ac:dyDescent="0.25">
@@ -3585,7 +3585,7 @@
         <v>155</v>
       </c>
       <c r="F79">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="80" spans="2:6" x14ac:dyDescent="0.25">
@@ -3602,7 +3602,7 @@
         <v>157</v>
       </c>
       <c r="F80">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="81" spans="2:6" x14ac:dyDescent="0.25">
@@ -3619,7 +3619,7 @@
         <v>159</v>
       </c>
       <c r="F81">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="82" spans="2:6" x14ac:dyDescent="0.25">
@@ -3636,7 +3636,7 @@
         <v>161</v>
       </c>
       <c r="F82">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="83" spans="2:6" x14ac:dyDescent="0.25">
@@ -3653,7 +3653,7 @@
         <v>163</v>
       </c>
       <c r="F83">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="84" spans="2:6" x14ac:dyDescent="0.25">
@@ -3670,7 +3670,7 @@
         <v>165</v>
       </c>
       <c r="F84">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="85" spans="2:6" x14ac:dyDescent="0.25">
@@ -3687,7 +3687,7 @@
         <v>167</v>
       </c>
       <c r="F85">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="86" spans="2:6" x14ac:dyDescent="0.25">
@@ -3704,7 +3704,7 @@
         <v>169</v>
       </c>
       <c r="F86">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="87" spans="2:6" x14ac:dyDescent="0.25">
@@ -3721,7 +3721,7 @@
         <v>171</v>
       </c>
       <c r="F87">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="88" spans="2:6" x14ac:dyDescent="0.25">
@@ -3738,7 +3738,7 @@
         <v>173</v>
       </c>
       <c r="F88">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="89" spans="2:6" x14ac:dyDescent="0.25">
@@ -3755,7 +3755,7 @@
         <v>175</v>
       </c>
       <c r="F89">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="90" spans="2:6" x14ac:dyDescent="0.25">
@@ -3772,7 +3772,7 @@
         <v>177</v>
       </c>
       <c r="F90">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="91" spans="2:6" x14ac:dyDescent="0.25">
@@ -3789,7 +3789,7 @@
         <v>179</v>
       </c>
       <c r="F91">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="92" spans="2:6" x14ac:dyDescent="0.25">
@@ -3806,7 +3806,7 @@
         <v>181</v>
       </c>
       <c r="F92">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="93" spans="2:6" x14ac:dyDescent="0.25">
@@ -3823,7 +3823,7 @@
         <v>183</v>
       </c>
       <c r="F93">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="94" spans="2:6" x14ac:dyDescent="0.25">
@@ -3840,7 +3840,7 @@
         <v>185</v>
       </c>
       <c r="F94">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="95" spans="2:6" x14ac:dyDescent="0.25">
@@ -3857,7 +3857,7 @@
         <v>107</v>
       </c>
       <c r="F95">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="96" spans="2:6" x14ac:dyDescent="0.25">
@@ -3874,7 +3874,7 @@
         <v>393</v>
       </c>
       <c r="F96">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="97" spans="2:6" x14ac:dyDescent="0.25">
@@ -3891,7 +3891,7 @@
         <v>187</v>
       </c>
       <c r="F97">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="98" spans="2:6" x14ac:dyDescent="0.25">
@@ -3908,7 +3908,7 @@
         <v>189</v>
       </c>
       <c r="F98">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="99" spans="2:6" x14ac:dyDescent="0.25">
@@ -3925,7 +3925,7 @@
         <v>149</v>
       </c>
       <c r="F99">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="100" spans="2:6" x14ac:dyDescent="0.25">
@@ -3942,7 +3942,7 @@
         <v>191</v>
       </c>
       <c r="F100">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="101" spans="2:6" x14ac:dyDescent="0.25">
@@ -3959,7 +3959,7 @@
         <v>193</v>
       </c>
       <c r="F101">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="102" spans="2:6" x14ac:dyDescent="0.25">
@@ -3976,7 +3976,7 @@
         <v>195</v>
       </c>
       <c r="F102">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="103" spans="2:6" x14ac:dyDescent="0.25">
@@ -3993,7 +3993,7 @@
         <v>197</v>
       </c>
       <c r="F103">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="104" spans="2:6" x14ac:dyDescent="0.25">
@@ -4010,7 +4010,7 @@
         <v>199</v>
       </c>
       <c r="F104">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="105" spans="2:6" x14ac:dyDescent="0.25">
@@ -4027,7 +4027,7 @@
         <v>201</v>
       </c>
       <c r="F105">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="106" spans="2:6" x14ac:dyDescent="0.25">
@@ -4044,7 +4044,7 @@
         <v>203</v>
       </c>
       <c r="F106">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="107" spans="2:6" x14ac:dyDescent="0.25">
@@ -4061,7 +4061,7 @@
         <v>205</v>
       </c>
       <c r="F107">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="108" spans="2:6" x14ac:dyDescent="0.25">
@@ -4078,7 +4078,7 @@
         <v>207</v>
       </c>
       <c r="F108">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="109" spans="2:6" x14ac:dyDescent="0.25">
@@ -4095,7 +4095,7 @@
         <v>209</v>
       </c>
       <c r="F109">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="110" spans="2:6" x14ac:dyDescent="0.25">
@@ -4112,7 +4112,7 @@
         <v>211</v>
       </c>
       <c r="F110">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="111" spans="2:6" x14ac:dyDescent="0.25">
@@ -4129,7 +4129,7 @@
         <v>213</v>
       </c>
       <c r="F111">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="112" spans="2:6" x14ac:dyDescent="0.25">
@@ -4146,7 +4146,7 @@
         <v>215</v>
       </c>
       <c r="F112">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="113" spans="2:6" x14ac:dyDescent="0.25">
@@ -4163,7 +4163,7 @@
         <v>217</v>
       </c>
       <c r="F113">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="114" spans="2:6" x14ac:dyDescent="0.25">
@@ -4180,7 +4180,7 @@
         <v>219</v>
       </c>
       <c r="F114">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="115" spans="2:6" x14ac:dyDescent="0.25">
@@ -4197,7 +4197,7 @@
         <v>221</v>
       </c>
       <c r="F115">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="116" spans="2:6" x14ac:dyDescent="0.25">
@@ -4214,7 +4214,7 @@
         <v>223</v>
       </c>
       <c r="F116">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="117" spans="2:6" x14ac:dyDescent="0.25">
@@ -4231,7 +4231,7 @@
         <v>225</v>
       </c>
       <c r="F117">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="118" spans="2:6" x14ac:dyDescent="0.25">
@@ -4248,7 +4248,7 @@
         <v>226</v>
       </c>
       <c r="F118">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="119" spans="2:6" x14ac:dyDescent="0.25">
@@ -4265,7 +4265,7 @@
         <v>228</v>
       </c>
       <c r="F119">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="120" spans="2:6" x14ac:dyDescent="0.25">
@@ -4282,7 +4282,7 @@
         <v>230</v>
       </c>
       <c r="F120">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="121" spans="2:6" x14ac:dyDescent="0.25">
@@ -4299,7 +4299,7 @@
         <v>232</v>
       </c>
       <c r="F121">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="122" spans="2:6" x14ac:dyDescent="0.25">
@@ -4316,7 +4316,7 @@
         <v>234</v>
       </c>
       <c r="F122">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="123" spans="2:6" x14ac:dyDescent="0.25">
@@ -4333,7 +4333,7 @@
         <v>236</v>
       </c>
       <c r="F123">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="124" spans="2:6" x14ac:dyDescent="0.25">
@@ -4350,7 +4350,7 @@
         <v>238</v>
       </c>
       <c r="F124">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="125" spans="2:6" x14ac:dyDescent="0.25">
@@ -4367,7 +4367,7 @@
         <v>240</v>
       </c>
       <c r="F125">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="126" spans="2:6" x14ac:dyDescent="0.25">
@@ -4384,7 +4384,7 @@
         <v>242</v>
       </c>
       <c r="F126">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="127" spans="2:6" x14ac:dyDescent="0.25">
@@ -4401,7 +4401,7 @@
         <v>244</v>
       </c>
       <c r="F127">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="128" spans="2:6" x14ac:dyDescent="0.25">
@@ -4418,7 +4418,7 @@
         <v>246</v>
       </c>
       <c r="F128">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="129" spans="2:6" x14ac:dyDescent="0.25">
@@ -4435,7 +4435,7 @@
         <v>248</v>
       </c>
       <c r="F129">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="130" spans="2:6" x14ac:dyDescent="0.25">
@@ -4452,7 +4452,7 @@
         <v>250</v>
       </c>
       <c r="F130">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="131" spans="2:6" x14ac:dyDescent="0.25">
@@ -4469,7 +4469,7 @@
         <v>252</v>
       </c>
       <c r="F131">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="132" spans="2:6" x14ac:dyDescent="0.25">
@@ -4486,7 +4486,7 @@
         <v>254</v>
       </c>
       <c r="F132">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="133" spans="2:6" x14ac:dyDescent="0.25">
@@ -4503,7 +4503,7 @@
         <v>256</v>
       </c>
       <c r="F133">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="134" spans="2:6" x14ac:dyDescent="0.25">
@@ -4520,7 +4520,7 @@
         <v>258</v>
       </c>
       <c r="F134">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="135" spans="2:6" x14ac:dyDescent="0.25">
@@ -4537,7 +4537,7 @@
         <v>260</v>
       </c>
       <c r="F135">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="136" spans="2:6" x14ac:dyDescent="0.25">
@@ -4554,7 +4554,7 @@
         <v>262</v>
       </c>
       <c r="F136">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="137" spans="2:6" x14ac:dyDescent="0.25">
@@ -4571,7 +4571,7 @@
         <v>264</v>
       </c>
       <c r="F137">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="138" spans="2:6" x14ac:dyDescent="0.25">
@@ -4588,7 +4588,7 @@
         <v>266</v>
       </c>
       <c r="F138">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="139" spans="2:6" x14ac:dyDescent="0.25">
@@ -4605,7 +4605,7 @@
         <v>268</v>
       </c>
       <c r="F139">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="140" spans="2:6" x14ac:dyDescent="0.25">
@@ -4622,7 +4622,7 @@
         <v>270</v>
       </c>
       <c r="F140">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="141" spans="2:6" x14ac:dyDescent="0.25">
@@ -4639,7 +4639,7 @@
         <v>272</v>
       </c>
       <c r="F141">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="142" spans="2:6" x14ac:dyDescent="0.25">
@@ -4656,7 +4656,7 @@
         <v>274</v>
       </c>
       <c r="F142">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="143" spans="2:6" x14ac:dyDescent="0.25">
@@ -4673,7 +4673,7 @@
         <v>276</v>
       </c>
       <c r="F143">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="144" spans="2:6" x14ac:dyDescent="0.25">
@@ -4690,7 +4690,7 @@
         <v>278</v>
       </c>
       <c r="F144">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="145" spans="2:6" x14ac:dyDescent="0.25">
@@ -4707,7 +4707,7 @@
         <v>280</v>
       </c>
       <c r="F145">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="146" spans="2:6" x14ac:dyDescent="0.25">
@@ -4724,7 +4724,7 @@
         <v>282</v>
       </c>
       <c r="F146">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="147" spans="2:6" x14ac:dyDescent="0.25">
@@ -4741,7 +4741,7 @@
         <v>284</v>
       </c>
       <c r="F147">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="148" spans="2:6" x14ac:dyDescent="0.25">
@@ -4758,7 +4758,7 @@
         <v>286</v>
       </c>
       <c r="F148">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="149" spans="2:6" x14ac:dyDescent="0.25">
@@ -4775,7 +4775,7 @@
         <v>288</v>
       </c>
       <c r="F149">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="150" spans="2:6" x14ac:dyDescent="0.25">
@@ -4792,7 +4792,7 @@
         <v>290</v>
       </c>
       <c r="F150">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="151" spans="2:6" x14ac:dyDescent="0.25">
@@ -4809,7 +4809,7 @@
         <v>292</v>
       </c>
       <c r="F151">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="152" spans="2:6" x14ac:dyDescent="0.25">
@@ -4826,7 +4826,7 @@
         <v>294</v>
       </c>
       <c r="F152">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="153" spans="2:6" x14ac:dyDescent="0.25">
@@ -4843,7 +4843,7 @@
         <v>296</v>
       </c>
       <c r="F153">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="154" spans="2:6" x14ac:dyDescent="0.25">
@@ -4860,7 +4860,7 @@
         <v>298</v>
       </c>
       <c r="F154">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="155" spans="2:6" x14ac:dyDescent="0.25">
@@ -4877,7 +4877,7 @@
         <v>300</v>
       </c>
       <c r="F155">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="156" spans="2:6" x14ac:dyDescent="0.25">
@@ -4894,7 +4894,7 @@
         <v>302</v>
       </c>
       <c r="F156">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="157" spans="2:6" x14ac:dyDescent="0.25">
@@ -4911,7 +4911,7 @@
         <v>303</v>
       </c>
       <c r="F157">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="158" spans="2:6" x14ac:dyDescent="0.25">
@@ -4928,7 +4928,7 @@
         <v>305</v>
       </c>
       <c r="F158">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="159" spans="2:6" x14ac:dyDescent="0.25">
@@ -4945,7 +4945,7 @@
         <v>307</v>
       </c>
       <c r="F159">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="160" spans="2:6" x14ac:dyDescent="0.25">
@@ -4962,7 +4962,7 @@
         <v>309</v>
       </c>
       <c r="F160">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="161" spans="2:6" x14ac:dyDescent="0.25">
@@ -4979,7 +4979,7 @@
         <v>615</v>
       </c>
       <c r="F161">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="162" spans="2:6" x14ac:dyDescent="0.25">
@@ -4996,7 +4996,7 @@
         <v>311</v>
       </c>
       <c r="F162">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="163" spans="2:6" x14ac:dyDescent="0.25">
@@ -5013,7 +5013,7 @@
         <v>313</v>
       </c>
       <c r="F163">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="164" spans="2:6" x14ac:dyDescent="0.25">
@@ -5030,7 +5030,7 @@
         <v>315</v>
       </c>
       <c r="F164">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="165" spans="2:6" x14ac:dyDescent="0.25">
@@ -5047,7 +5047,7 @@
         <v>317</v>
       </c>
       <c r="F165">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="166" spans="2:6" x14ac:dyDescent="0.25">
@@ -5064,7 +5064,7 @@
         <v>319</v>
       </c>
       <c r="F166">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="167" spans="2:6" x14ac:dyDescent="0.25">
@@ -5081,7 +5081,7 @@
         <v>321</v>
       </c>
       <c r="F167">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="168" spans="2:6" x14ac:dyDescent="0.25">
@@ -5098,7 +5098,7 @@
         <v>323</v>
       </c>
       <c r="F168">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="169" spans="2:6" x14ac:dyDescent="0.25">
@@ -5115,7 +5115,7 @@
         <v>325</v>
       </c>
       <c r="F169">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="170" spans="2:6" x14ac:dyDescent="0.25">
@@ -5132,7 +5132,7 @@
         <v>327</v>
       </c>
       <c r="F170">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="171" spans="2:6" x14ac:dyDescent="0.25">
@@ -5149,7 +5149,7 @@
         <v>329</v>
       </c>
       <c r="F171">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="172" spans="2:6" x14ac:dyDescent="0.25">
@@ -5166,7 +5166,7 @@
         <v>331</v>
       </c>
       <c r="F172">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="173" spans="2:6" x14ac:dyDescent="0.25">
@@ -5183,7 +5183,7 @@
         <v>333</v>
       </c>
       <c r="F173">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="174" spans="2:6" x14ac:dyDescent="0.25">
@@ -5200,7 +5200,7 @@
         <v>335</v>
       </c>
       <c r="F174">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="175" spans="2:6" x14ac:dyDescent="0.25">
@@ -5217,7 +5217,7 @@
         <v>337</v>
       </c>
       <c r="F175">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="176" spans="2:6" x14ac:dyDescent="0.25">
@@ -5234,7 +5234,7 @@
         <v>339</v>
       </c>
       <c r="F176">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="177" spans="2:6" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>341</v>
       </c>
       <c r="F177">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="178" spans="2:6" x14ac:dyDescent="0.25">
@@ -5268,7 +5268,7 @@
         <v>343</v>
       </c>
       <c r="F178">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="179" spans="2:6" x14ac:dyDescent="0.25">
@@ -5285,7 +5285,7 @@
         <v>345</v>
       </c>
       <c r="F179">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="180" spans="2:6" x14ac:dyDescent="0.25">
@@ -5302,7 +5302,7 @@
         <v>347</v>
       </c>
       <c r="F180">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="181" spans="2:6" x14ac:dyDescent="0.25">
@@ -5319,7 +5319,7 @@
         <v>349</v>
       </c>
       <c r="F181">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="182" spans="2:6" x14ac:dyDescent="0.25">
@@ -5336,7 +5336,7 @@
         <v>351</v>
       </c>
       <c r="F182">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="183" spans="2:6" x14ac:dyDescent="0.25">
@@ -5353,7 +5353,7 @@
         <v>353</v>
       </c>
       <c r="F183">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="184" spans="2:6" x14ac:dyDescent="0.25">
@@ -5370,7 +5370,7 @@
         <v>355</v>
       </c>
       <c r="F184">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="185" spans="2:6" x14ac:dyDescent="0.25">
@@ -5387,7 +5387,7 @@
         <v>357</v>
       </c>
       <c r="F185">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="186" spans="2:6" x14ac:dyDescent="0.25">
@@ -5404,7 +5404,7 @@
         <v>359</v>
       </c>
       <c r="F186">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="187" spans="2:6" x14ac:dyDescent="0.25">
@@ -5421,7 +5421,7 @@
         <v>361</v>
       </c>
       <c r="F187">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="188" spans="2:6" x14ac:dyDescent="0.25">
@@ -5438,7 +5438,7 @@
         <v>363</v>
       </c>
       <c r="F188">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="189" spans="2:6" x14ac:dyDescent="0.25">
@@ -5455,7 +5455,7 @@
         <v>365</v>
       </c>
       <c r="F189">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="190" spans="2:6" x14ac:dyDescent="0.25">
@@ -5472,7 +5472,7 @@
         <v>367</v>
       </c>
       <c r="F190">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="191" spans="2:6" x14ac:dyDescent="0.25">
@@ -5489,7 +5489,7 @@
         <v>369</v>
       </c>
       <c r="F191">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="192" spans="2:6" x14ac:dyDescent="0.25">
@@ -5506,7 +5506,7 @@
         <v>371</v>
       </c>
       <c r="F192">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="193" spans="2:6" x14ac:dyDescent="0.25">
@@ -5523,7 +5523,7 @@
         <v>373</v>
       </c>
       <c r="F193">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="194" spans="2:6" x14ac:dyDescent="0.25">
@@ -5540,7 +5540,7 @@
         <v>375</v>
       </c>
       <c r="F194">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="195" spans="2:6" x14ac:dyDescent="0.25">
@@ -5557,7 +5557,7 @@
         <v>109</v>
       </c>
       <c r="F195">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="196" spans="2:6" x14ac:dyDescent="0.25">
@@ -5574,7 +5574,7 @@
         <v>185</v>
       </c>
       <c r="F196">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="197" spans="2:6" x14ac:dyDescent="0.25">
@@ -5591,7 +5591,7 @@
         <v>378</v>
       </c>
       <c r="F197">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="198" spans="2:6" x14ac:dyDescent="0.25">
@@ -5608,7 +5608,7 @@
         <v>380</v>
       </c>
       <c r="F198">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="199" spans="2:6" x14ac:dyDescent="0.25">
@@ -5625,7 +5625,7 @@
         <v>382</v>
       </c>
       <c r="F199">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="200" spans="2:6" x14ac:dyDescent="0.25">
@@ -5642,7 +5642,7 @@
         <v>384</v>
       </c>
       <c r="F200">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="201" spans="2:6" x14ac:dyDescent="0.25">
@@ -5659,7 +5659,7 @@
         <v>386</v>
       </c>
       <c r="F201">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="202" spans="2:6" x14ac:dyDescent="0.25">
@@ -5676,7 +5676,7 @@
         <v>389</v>
       </c>
       <c r="F202">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="203" spans="2:6" x14ac:dyDescent="0.25">
@@ -5693,7 +5693,7 @@
         <v>391</v>
       </c>
       <c r="F203">
-        <v>47</v>
+        <v>408</v>
       </c>
     </row>
     <row r="204" spans="2:6" x14ac:dyDescent="0.25">
@@ -5710,7 +5710,7 @@
         <v>504</v>
       </c>
       <c r="F204">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="205" spans="2:6" x14ac:dyDescent="0.25">
@@ -5727,7 +5727,7 @@
         <v>505</v>
       </c>
       <c r="F205">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="206" spans="2:6" x14ac:dyDescent="0.25">
@@ -5744,7 +5744,7 @@
         <v>506</v>
       </c>
       <c r="F206">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="207" spans="2:6" x14ac:dyDescent="0.25">
@@ -5761,7 +5761,7 @@
         <v>507</v>
       </c>
       <c r="F207">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="208" spans="2:6" x14ac:dyDescent="0.25">
@@ -5778,7 +5778,7 @@
         <v>508</v>
       </c>
       <c r="F208">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="209" spans="2:6" x14ac:dyDescent="0.25">
@@ -5795,7 +5795,7 @@
         <v>509</v>
       </c>
       <c r="F209">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="210" spans="2:6" x14ac:dyDescent="0.25">
@@ -5812,7 +5812,7 @@
         <v>510</v>
       </c>
       <c r="F210">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="211" spans="2:6" x14ac:dyDescent="0.25">
@@ -5829,7 +5829,7 @@
         <v>511</v>
       </c>
       <c r="F211">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="212" spans="2:6" x14ac:dyDescent="0.25">
@@ -5846,7 +5846,7 @@
         <v>512</v>
       </c>
       <c r="F212">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="213" spans="2:6" x14ac:dyDescent="0.25">
@@ -5863,7 +5863,7 @@
         <v>513</v>
       </c>
       <c r="F213">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="214" spans="2:6" x14ac:dyDescent="0.25">
@@ -5880,7 +5880,7 @@
         <v>514</v>
       </c>
       <c r="F214">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="215" spans="2:6" x14ac:dyDescent="0.25">
@@ -5897,7 +5897,7 @@
         <v>515</v>
       </c>
       <c r="F215">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="216" spans="2:6" x14ac:dyDescent="0.25">
@@ -5914,7 +5914,7 @@
         <v>516</v>
       </c>
       <c r="F216">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="217" spans="2:6" x14ac:dyDescent="0.25">
@@ -5931,7 +5931,7 @@
         <v>517</v>
       </c>
       <c r="F217">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="218" spans="2:6" x14ac:dyDescent="0.25">
@@ -5948,7 +5948,7 @@
         <v>518</v>
       </c>
       <c r="F218">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="219" spans="2:6" x14ac:dyDescent="0.25">
@@ -5965,7 +5965,7 @@
         <v>519</v>
       </c>
       <c r="F219">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="220" spans="2:6" x14ac:dyDescent="0.25">
@@ -5982,7 +5982,7 @@
         <v>520</v>
       </c>
       <c r="F220">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="221" spans="2:6" x14ac:dyDescent="0.25">
@@ -5999,7 +5999,7 @@
         <v>521</v>
       </c>
       <c r="F221">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="222" spans="2:6" x14ac:dyDescent="0.25">
@@ -6016,7 +6016,7 @@
         <v>522</v>
       </c>
       <c r="F222">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="223" spans="2:6" x14ac:dyDescent="0.25">
@@ -6033,7 +6033,7 @@
         <v>523</v>
       </c>
       <c r="F223">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="224" spans="2:6" x14ac:dyDescent="0.25">
@@ -6050,7 +6050,7 @@
         <v>524</v>
       </c>
       <c r="F224">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="225" spans="2:6" x14ac:dyDescent="0.25">
@@ -6067,7 +6067,7 @@
         <v>525</v>
       </c>
       <c r="F225">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="226" spans="2:6" x14ac:dyDescent="0.25">
@@ -6084,7 +6084,7 @@
         <v>526</v>
       </c>
       <c r="F226">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="227" spans="2:6" x14ac:dyDescent="0.25">
@@ -6101,7 +6101,7 @@
         <v>527</v>
       </c>
       <c r="F227">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="228" spans="2:6" x14ac:dyDescent="0.25">
@@ -6118,7 +6118,7 @@
         <v>528</v>
       </c>
       <c r="F228">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="229" spans="2:6" x14ac:dyDescent="0.25">
@@ -6135,7 +6135,7 @@
         <v>529</v>
       </c>
       <c r="F229">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="230" spans="2:6" x14ac:dyDescent="0.25">
@@ -6152,7 +6152,7 @@
         <v>530</v>
       </c>
       <c r="F230">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="231" spans="2:6" x14ac:dyDescent="0.25">
@@ -6169,7 +6169,7 @@
         <v>531</v>
       </c>
       <c r="F231">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="232" spans="2:6" x14ac:dyDescent="0.25">
@@ -6186,7 +6186,7 @@
         <v>532</v>
       </c>
       <c r="F232">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="233" spans="2:6" x14ac:dyDescent="0.25">
@@ -6203,7 +6203,7 @@
         <v>533</v>
       </c>
       <c r="F233">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="234" spans="2:6" x14ac:dyDescent="0.25">
@@ -6220,7 +6220,7 @@
         <v>534</v>
       </c>
       <c r="F234">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="235" spans="2:6" x14ac:dyDescent="0.25">
@@ -6237,7 +6237,7 @@
         <v>535</v>
       </c>
       <c r="F235">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="236" spans="2:6" x14ac:dyDescent="0.25">
@@ -6254,7 +6254,7 @@
         <v>536</v>
       </c>
       <c r="F236">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="237" spans="2:6" x14ac:dyDescent="0.25">
@@ -6271,7 +6271,7 @@
         <v>537</v>
       </c>
       <c r="F237">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="238" spans="2:6" x14ac:dyDescent="0.25">
@@ -6288,7 +6288,7 @@
         <v>538</v>
       </c>
       <c r="F238">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="239" spans="2:6" x14ac:dyDescent="0.25">
@@ -6305,7 +6305,7 @@
         <v>539</v>
       </c>
       <c r="F239">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="240" spans="2:6" x14ac:dyDescent="0.25">
@@ -6322,7 +6322,7 @@
         <v>540</v>
       </c>
       <c r="F240">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="241" spans="2:6" x14ac:dyDescent="0.25">
@@ -6339,7 +6339,7 @@
         <v>541</v>
       </c>
       <c r="F241">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="242" spans="2:6" x14ac:dyDescent="0.25">
@@ -6356,7 +6356,7 @@
         <v>433</v>
       </c>
       <c r="F242">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="243" spans="2:6" x14ac:dyDescent="0.25">
@@ -6373,7 +6373,7 @@
         <v>542</v>
       </c>
       <c r="F243">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="244" spans="2:6" x14ac:dyDescent="0.25">
@@ -6390,7 +6390,7 @@
         <v>151</v>
       </c>
       <c r="F244">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="245" spans="2:6" x14ac:dyDescent="0.25">
@@ -6407,7 +6407,7 @@
         <v>543</v>
       </c>
       <c r="F245">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="246" spans="2:6" x14ac:dyDescent="0.25">
@@ -6424,7 +6424,7 @@
         <v>544</v>
       </c>
       <c r="F246">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="247" spans="2:6" x14ac:dyDescent="0.25">
@@ -6441,7 +6441,7 @@
         <v>545</v>
       </c>
       <c r="F247">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="248" spans="2:6" x14ac:dyDescent="0.25">
@@ -6458,7 +6458,7 @@
         <v>546</v>
       </c>
       <c r="F248">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="249" spans="2:6" x14ac:dyDescent="0.25">
@@ -6475,7 +6475,7 @@
         <v>547</v>
       </c>
       <c r="F249">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="250" spans="2:6" x14ac:dyDescent="0.25">
@@ -6492,7 +6492,7 @@
         <v>548</v>
       </c>
       <c r="F250">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="251" spans="2:6" x14ac:dyDescent="0.25">
@@ -6509,7 +6509,7 @@
         <v>549</v>
       </c>
       <c r="F251">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="252" spans="2:6" x14ac:dyDescent="0.25">
@@ -6526,7 +6526,7 @@
         <v>550</v>
       </c>
       <c r="F252">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="253" spans="2:6" x14ac:dyDescent="0.25">
@@ -6543,7 +6543,7 @@
         <v>551</v>
       </c>
       <c r="F253">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="254" spans="2:6" x14ac:dyDescent="0.25">
@@ -6560,7 +6560,7 @@
         <v>552</v>
       </c>
       <c r="F254">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="255" spans="2:6" x14ac:dyDescent="0.25">
@@ -6577,7 +6577,7 @@
         <v>553</v>
       </c>
       <c r="F255">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="256" spans="2:6" x14ac:dyDescent="0.25">
@@ -6594,7 +6594,7 @@
         <v>554</v>
       </c>
       <c r="F256">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="257" spans="2:6" x14ac:dyDescent="0.25">
@@ -6611,7 +6611,7 @@
         <v>555</v>
       </c>
       <c r="F257">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="258" spans="2:6" x14ac:dyDescent="0.25">
@@ -6628,7 +6628,7 @@
         <v>556</v>
       </c>
       <c r="F258">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="259" spans="2:6" x14ac:dyDescent="0.25">
@@ -6645,7 +6645,7 @@
         <v>557</v>
       </c>
       <c r="F259">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="260" spans="2:6" x14ac:dyDescent="0.25">
@@ -6662,7 +6662,7 @@
         <v>558</v>
       </c>
       <c r="F260">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="261" spans="2:6" x14ac:dyDescent="0.25">
@@ -6679,7 +6679,7 @@
         <v>559</v>
       </c>
       <c r="F261">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="262" spans="2:6" x14ac:dyDescent="0.25">
@@ -6696,7 +6696,7 @@
         <v>560</v>
       </c>
       <c r="F262">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="263" spans="2:6" x14ac:dyDescent="0.25">
@@ -6713,7 +6713,7 @@
         <v>561</v>
       </c>
       <c r="F263">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="264" spans="2:6" x14ac:dyDescent="0.25">
@@ -6730,7 +6730,7 @@
         <v>562</v>
       </c>
       <c r="F264">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="265" spans="2:6" x14ac:dyDescent="0.25">
@@ -6747,7 +6747,7 @@
         <v>563</v>
       </c>
       <c r="F265">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="266" spans="2:6" x14ac:dyDescent="0.25">
@@ -6764,7 +6764,7 @@
         <v>564</v>
       </c>
       <c r="F266">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="267" spans="2:6" x14ac:dyDescent="0.25">
@@ -6781,7 +6781,7 @@
         <v>565</v>
       </c>
       <c r="F267">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="268" spans="2:6" x14ac:dyDescent="0.25">
@@ -6798,7 +6798,7 @@
         <v>566</v>
       </c>
       <c r="F268">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="269" spans="2:6" x14ac:dyDescent="0.25">
@@ -6815,7 +6815,7 @@
         <v>567</v>
       </c>
       <c r="F269">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="270" spans="2:6" x14ac:dyDescent="0.25">
@@ -6832,7 +6832,7 @@
         <v>568</v>
       </c>
       <c r="F270">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="271" spans="2:6" x14ac:dyDescent="0.25">
@@ -6849,7 +6849,7 @@
         <v>569</v>
       </c>
       <c r="F271">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="272" spans="2:6" x14ac:dyDescent="0.25">
@@ -6866,7 +6866,7 @@
         <v>570</v>
       </c>
       <c r="F272">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="273" spans="2:6" x14ac:dyDescent="0.25">
@@ -6883,7 +6883,7 @@
         <v>571</v>
       </c>
       <c r="F273">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="274" spans="2:6" x14ac:dyDescent="0.25">
@@ -6900,7 +6900,7 @@
         <v>572</v>
       </c>
       <c r="F274">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="275" spans="2:6" x14ac:dyDescent="0.25">
@@ -6917,7 +6917,7 @@
         <v>573</v>
       </c>
       <c r="F275">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="276" spans="2:6" x14ac:dyDescent="0.25">
@@ -6934,7 +6934,7 @@
         <v>574</v>
       </c>
       <c r="F276">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="277" spans="2:6" x14ac:dyDescent="0.25">
@@ -6951,7 +6951,7 @@
         <v>575</v>
       </c>
       <c r="F277">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="278" spans="2:6" x14ac:dyDescent="0.25">
@@ -6968,7 +6968,7 @@
         <v>576</v>
       </c>
       <c r="F278">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="279" spans="2:6" x14ac:dyDescent="0.25">
@@ -6985,7 +6985,7 @@
         <v>577</v>
       </c>
       <c r="F279">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="280" spans="2:6" x14ac:dyDescent="0.25">
@@ -7002,7 +7002,7 @@
         <v>578</v>
       </c>
       <c r="F280">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="281" spans="2:6" x14ac:dyDescent="0.25">
@@ -7019,7 +7019,7 @@
         <v>579</v>
       </c>
       <c r="F281">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="282" spans="2:6" x14ac:dyDescent="0.25">
@@ -7036,7 +7036,7 @@
         <v>580</v>
       </c>
       <c r="F282">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="283" spans="2:6" x14ac:dyDescent="0.25">
@@ -7053,7 +7053,7 @@
         <v>581</v>
       </c>
       <c r="F283">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="284" spans="2:6" x14ac:dyDescent="0.25">
@@ -7070,7 +7070,7 @@
         <v>582</v>
       </c>
       <c r="F284">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="285" spans="2:6" x14ac:dyDescent="0.25">
@@ -7087,7 +7087,7 @@
         <v>583</v>
       </c>
       <c r="F285">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="286" spans="2:6" x14ac:dyDescent="0.25">
@@ -7104,7 +7104,7 @@
         <v>584</v>
       </c>
       <c r="F286">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="287" spans="2:6" x14ac:dyDescent="0.25">
@@ -7121,7 +7121,7 @@
         <v>159</v>
       </c>
       <c r="F287">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="288" spans="2:6" x14ac:dyDescent="0.25">
@@ -7138,7 +7138,7 @@
         <v>474</v>
       </c>
       <c r="F288">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="289" spans="2:6" x14ac:dyDescent="0.25">
@@ -7155,7 +7155,7 @@
         <v>585</v>
       </c>
       <c r="F289">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="290" spans="2:6" x14ac:dyDescent="0.25">
@@ -7172,7 +7172,7 @@
         <v>586</v>
       </c>
       <c r="F290">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="291" spans="2:6" x14ac:dyDescent="0.25">
@@ -7189,7 +7189,7 @@
         <v>587</v>
       </c>
       <c r="F291">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="292" spans="2:6" x14ac:dyDescent="0.25">
@@ -7206,7 +7206,7 @@
         <v>588</v>
       </c>
       <c r="F292">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="293" spans="2:6" x14ac:dyDescent="0.25">
@@ -7223,7 +7223,7 @@
         <v>589</v>
       </c>
       <c r="F293">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="294" spans="2:6" x14ac:dyDescent="0.25">
@@ -7240,7 +7240,7 @@
         <v>590</v>
       </c>
       <c r="F294">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="295" spans="2:6" x14ac:dyDescent="0.25">
@@ -7257,7 +7257,7 @@
         <v>591</v>
       </c>
       <c r="F295">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="296" spans="2:6" x14ac:dyDescent="0.25">
@@ -7274,7 +7274,7 @@
         <v>592</v>
       </c>
       <c r="F296">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="297" spans="2:6" x14ac:dyDescent="0.25">
@@ -7291,7 +7291,7 @@
         <v>593</v>
       </c>
       <c r="F297">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="298" spans="2:6" x14ac:dyDescent="0.25">
@@ -7308,7 +7308,7 @@
         <v>594</v>
       </c>
       <c r="F298">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="299" spans="2:6" x14ac:dyDescent="0.25">
@@ -7325,7 +7325,7 @@
         <v>595</v>
       </c>
       <c r="F299">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="300" spans="2:6" x14ac:dyDescent="0.25">
@@ -7342,7 +7342,7 @@
         <v>596</v>
       </c>
       <c r="F300">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="301" spans="2:6" x14ac:dyDescent="0.25">
@@ -7359,7 +7359,7 @@
         <v>597</v>
       </c>
       <c r="F301">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="302" spans="2:6" x14ac:dyDescent="0.25">
@@ -7376,7 +7376,7 @@
         <v>598</v>
       </c>
       <c r="F302">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="303" spans="2:6" x14ac:dyDescent="0.25">
@@ -7393,7 +7393,7 @@
         <v>599</v>
       </c>
       <c r="F303">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="304" spans="2:6" x14ac:dyDescent="0.25">
@@ -7410,7 +7410,7 @@
         <v>600</v>
       </c>
       <c r="F304">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="305" spans="2:6" x14ac:dyDescent="0.25">
@@ -7427,7 +7427,7 @@
         <v>601</v>
       </c>
       <c r="F305">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="306" spans="2:6" x14ac:dyDescent="0.25">
@@ -7444,7 +7444,7 @@
         <v>602</v>
       </c>
       <c r="F306">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="307" spans="2:6" x14ac:dyDescent="0.25">
@@ -7461,7 +7461,7 @@
         <v>603</v>
       </c>
       <c r="F307">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="308" spans="2:6" x14ac:dyDescent="0.25">
@@ -7478,7 +7478,7 @@
         <v>604</v>
       </c>
       <c r="F308">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="309" spans="2:6" x14ac:dyDescent="0.25">
@@ -7495,7 +7495,7 @@
         <v>605</v>
       </c>
       <c r="F309">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="310" spans="2:6" x14ac:dyDescent="0.25">
@@ -7512,7 +7512,7 @@
         <v>606</v>
       </c>
       <c r="F310">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="311" spans="2:6" x14ac:dyDescent="0.25">
@@ -7529,7 +7529,7 @@
         <v>607</v>
       </c>
       <c r="F311">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="312" spans="2:6" x14ac:dyDescent="0.25">
@@ -7546,7 +7546,7 @@
         <v>608</v>
       </c>
       <c r="F312">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="313" spans="2:6" x14ac:dyDescent="0.25">
@@ -7563,7 +7563,7 @@
         <v>548</v>
       </c>
       <c r="F313">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="314" spans="2:6" x14ac:dyDescent="0.25">
@@ -7580,7 +7580,7 @@
         <v>609</v>
       </c>
       <c r="F314">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="315" spans="2:6" x14ac:dyDescent="0.25">
@@ -7597,7 +7597,7 @@
         <v>610</v>
       </c>
       <c r="F315">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="316" spans="2:6" x14ac:dyDescent="0.25">
@@ -7614,7 +7614,7 @@
         <v>611</v>
       </c>
       <c r="F316">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="317" spans="2:6" x14ac:dyDescent="0.25">
@@ -7631,7 +7631,7 @@
         <v>612</v>
       </c>
       <c r="F317">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
     <row r="318" spans="2:6" x14ac:dyDescent="0.25">
@@ -7648,7 +7648,7 @@
         <v>613</v>
       </c>
       <c r="F318">
-        <v>52</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>